<commit_message>
feat: reorder works and refresh favicon
</commit_message>
<xml_diff>
--- a/public/data/works.xlsx
+++ b/public/data/works.xlsx
@@ -791,7 +791,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="2">
         <is>
-          <t>ohir-brand-film</t>
+          <t>vfx-2026-showreel</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="2">
@@ -801,7 +801,7 @@
       </c>
       <c r="C20" t="inlineStr" s="2">
         <is>
-          <t>OHIR</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="2">
@@ -821,24 +821,24 @@
       </c>
       <c r="G20" t="inlineStr" s="2">
         <is>
-          <t>‘OHIR' BRAND FILM - FULL AI</t>
+          <t>Personal Work - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="2">
         <is>
-          <t>ohir-brand-filmalter</t>
+          <t>vfx-2026-kyuto-butterflyland</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="2">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="2">
         <is>
-          <t>OHIR</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="2">
@@ -858,14 +858,14 @@
       </c>
       <c r="G21" t="inlineStr" s="2">
         <is>
-          <t>‘OHIR' BRAND FILM(ALTERS) - FULL AI</t>
+          <t>[KYUTO TURNS 31 FILM #01] - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr" s="2">
         <is>
-          <t>poster-2026-kyuto31</t>
+          <t>vfx-2026-kyuto-rabbit</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="2">
@@ -875,12 +875,12 @@
       </c>
       <c r="C22" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="2">
@@ -895,14 +895,14 @@
       </c>
       <c r="G22" t="inlineStr" s="2">
         <is>
-          <t>BIRTHDAY VISUALS for KYUTO</t>
+          <t>[KYUTO TURNS 31 FILM #02] - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr" s="2">
         <is>
-          <t>poster-2025-kyuto30</t>
+          <t>vfx-2026-kyuto-cafe</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="2">
@@ -912,17 +912,17 @@
       </c>
       <c r="C23" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="2">
@@ -932,14 +932,14 @@
       </c>
       <c r="G23" t="inlineStr" s="2">
         <is>
-          <t>BIRTHDAY VISUALS for KYUTO</t>
+          <t>[KYUTO TURNS 31 FILM #03] - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr" s="2">
         <is>
-          <t>poster-2025-hanni</t>
+          <t>vfx-2026-aespaphoto</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="2">
@@ -949,17 +949,17 @@
       </c>
       <c r="C24" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="2">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="2">
@@ -969,14 +969,14 @@
       </c>
       <c r="G24" t="inlineStr" s="2">
         <is>
-          <t>BIRTHDAY VISUALS for JONGIN</t>
+          <t>[Aespa] - AUGMENTED FULL AI GRAPHIC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr" s="2">
         <is>
-          <t>album-cover-lack</t>
+          <t>vfx-2026-lunanewyear</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="2">
@@ -986,17 +986,17 @@
       </c>
       <c r="C25" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="2">
@@ -1006,34 +1006,34 @@
       </c>
       <c r="G25" t="inlineStr" s="2">
         <is>
-          <t>ALBUM COVER for LACK</t>
+          <t>[Lunar New Year] - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr" s="2">
         <is>
-          <t>album-cover-crane</t>
+          <t>vfx-2026-bangbang</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="2">
@@ -1043,14 +1043,14 @@
       </c>
       <c r="G26" t="inlineStr" s="2">
         <is>
-          <t>ALBUM COVER for CRANE</t>
+          <t>Personal Work - AI VFX</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr" s="2">
         <is>
-          <t>album-cover-laegyu</t>
+          <t>vfx-2026-lesserafim</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="2">
@@ -1060,17 +1060,17 @@
       </c>
       <c r="C27" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="2">
         <is>
-          <t>GRAPHIC</t>
+          <t>AI Works / 3D</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="2">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="2">
@@ -1080,19 +1080,19 @@
       </c>
       <c r="G27" t="inlineStr" s="2">
         <is>
-          <t>ALBUM COVER for LAEGYU</t>
+          <t>Personal Work - AI VFX</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-showreel</t>
+          <t>vfx-2026-newjeans</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="2">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="G28" t="inlineStr" s="2">
         <is>
-          <t>Personal Work - FULL AI</t>
+          <t>Personal Work - AI VFX</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-kyuto-butterflyland</t>
+          <t>vfx-2026-cortis-redred</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="2">
@@ -1154,19 +1154,19 @@
       </c>
       <c r="G29" t="inlineStr" s="2">
         <is>
-          <t>[KYUTO TURNS 31 FILM #01] - FULL AI</t>
+          <t>Personal Work - AI VFX</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-kyuto-rabbit</t>
+          <t>vfx-2026-iyodrama</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="2">
@@ -1191,19 +1191,19 @@
       </c>
       <c r="G30" t="inlineStr" s="2">
         <is>
-          <t>[KYUTO TURNS 31 FILM #02] - FULL AI</t>
+          <t>Personal Work - AI VFX</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-kyuto-cafe</t>
+          <t>vfx-2025-nike</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="2">
@@ -1228,19 +1228,19 @@
       </c>
       <c r="G31" t="inlineStr" s="2">
         <is>
-          <t>[KYUTO TURNS 31 FILM #03] - FULL AI</t>
+          <t>[NIKE] - FULL 3D</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-aespaphoto</t>
+          <t>vfx-2025-xg</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="2">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="E32" t="inlineStr" s="2">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="2">
@@ -1265,19 +1265,19 @@
       </c>
       <c r="G32" t="inlineStr" s="2">
         <is>
-          <t>[Aespa] - AUGMENTED FULL AI GRAPHIC</t>
+          <t>[Something Ain’t Right] - FULL 3D</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-lunanewyear</t>
+          <t>vfx-2025-aesop</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="2">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="E33" t="inlineStr" s="2">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="2">
@@ -1302,19 +1302,19 @@
       </c>
       <c r="G33" t="inlineStr" s="2">
         <is>
-          <t>[Lunar New Year] - FULL AI</t>
+          <t>[Aesop] - 3D Comp</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-bangbang</t>
+          <t>vfx-2025-kiiikiii</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="2">
         <is>
-          <t>false</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="2">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="E34" t="inlineStr" s="2">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="2">
@@ -1339,19 +1339,19 @@
       </c>
       <c r="G34" t="inlineStr" s="2">
         <is>
-          <t>Personal Work - AI VFX</t>
+          <t>[BTG] - FULL 3D</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-lesserafim</t>
+          <t>vfx-2025-vivienne</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="2">
         <is>
-          <t>false</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="2">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="E35" t="inlineStr" s="2">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="2">
@@ -1376,31 +1376,31 @@
       </c>
       <c r="G35" t="inlineStr" s="2">
         <is>
-          <t>Personal Work - AI VFX</t>
+          <t>[Vivienne Westwood] - FULL 3D</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-newjeans</t>
+          <t>ohir-brand-film</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="2">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="2">
         <is>
+          <t>OHIR</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr" s="2">
+        <is>
           <t>AI Works / 3D</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr" s="2">
-        <is>
-          <t>AI Works / 3D</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr" s="2">
         <is>
           <t>2026</t>
@@ -1413,31 +1413,31 @@
       </c>
       <c r="G36" t="inlineStr" s="2">
         <is>
-          <t>Personal Work - AI VFX</t>
+          <t>‘OHIR' BRAND FILM - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-cortis-redred</t>
+          <t>ohir-brand-filmalter</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="2">
         <is>
-          <t>false</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="2">
         <is>
+          <t>OHIR</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr" s="2">
+        <is>
           <t>AI Works / 3D</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr" s="2">
-        <is>
-          <t>AI Works / 3D</t>
-        </is>
-      </c>
       <c r="E37" t="inlineStr" s="2">
         <is>
           <t>2026</t>
@@ -1450,34 +1450,34 @@
       </c>
       <c r="G37" t="inlineStr" s="2">
         <is>
-          <t>Personal Work - AI VFX</t>
+          <t>‘OHIR' BRAND FILM(ALTERS) - FULL AI</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr" s="2">
         <is>
-          <t>vfx-2026-iyodrama</t>
+          <t>ojat-styling-01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="2">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>OJAT</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="2">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="2">
@@ -1487,34 +1487,34 @@
       </c>
       <c r="G38" t="inlineStr" s="2">
         <is>
-          <t>Personal Work - AI VFX</t>
+          <t>VISUAL DIRECTING for EDITORIAL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr" s="2">
         <is>
-          <t>vfx-2025-nike</t>
+          <t>ojat-lookbook-2021</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="2">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C39" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>OJAT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="2">
         <is>
-          <t>2026</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="2">
@@ -1524,34 +1524,34 @@
       </c>
       <c r="G39" t="inlineStr" s="2">
         <is>
-          <t>[NIKE] - FULL 3D</t>
+          <t>'OJAT' 21' LOOKBOOK</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr" s="2">
         <is>
-          <t>vfx-2025-xg</t>
+          <t>ojat-lookbook-2021-editorial</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="2">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>OJAT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="2">
@@ -1561,34 +1561,34 @@
       </c>
       <c r="G40" t="inlineStr" s="2">
         <is>
-          <t>[Something Ain’t Right] - FULL 3D</t>
+          <t>‘OJAT' 21' EDITORIAL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr" s="2">
         <is>
-          <t>vfx-2025-aesop</t>
+          <t>ojat-lookbook-2021-development</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="2">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>OJAT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="2">
@@ -1598,34 +1598,34 @@
       </c>
       <c r="G41" t="inlineStr" s="2">
         <is>
-          <t>[Aesop] - 3D Comp</t>
+          <t>‘OJAT' 21' DEVELOPMENT</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr" s="2">
         <is>
-          <t>vfx-2025-kiiikiii</t>
+          <t>ojat-lookbook-2020</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="2">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>OJAT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="2">
@@ -1635,34 +1635,34 @@
       </c>
       <c r="G42" t="inlineStr" s="2">
         <is>
-          <t>[BTG] - FULL 3D</t>
+          <t>‘OJAT' 20’ LOOKBOOK</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr" s="2">
         <is>
-          <t>vfx-2025-vivienne</t>
+          <t>ojat-lookbook-2020-editorial</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="2">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>OJAT</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="2">
         <is>
-          <t>AI Works / 3D</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="2">
         <is>
-          <t>2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="2">
@@ -1672,14 +1672,14 @@
       </c>
       <c r="G43" t="inlineStr" s="2">
         <is>
-          <t>[Vivienne Westwood] - FULL 3D</t>
+          <t>‘OJAT' 20’ EDITORIAL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr" s="2">
         <is>
-          <t>ojat-styling-01</t>
+          <t>ojat-lookbook-2020-development</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="2">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="E44" t="inlineStr" s="2">
         <is>
-          <t>2023</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="2">
@@ -1709,14 +1709,14 @@
       </c>
       <c r="G44" t="inlineStr" s="2">
         <is>
-          <t>VISUAL DIRECTING for EDITORIAL</t>
+          <t>‘OJAT' 20' DEVELOPMENT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr" s="2">
         <is>
-          <t>ojat-lookbook-2021</t>
+          <t>ojat-magazine-pap</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="2">
@@ -1746,14 +1746,14 @@
       </c>
       <c r="G45" t="inlineStr" s="2">
         <is>
-          <t>'OJAT' 21' LOOKBOOK</t>
+          <t>VISAUL for 'PAP Magazine' - In the Name of Love</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr" s="2">
         <is>
-          <t>ojat-lookbook-2021-editorial</t>
+          <t>ojat-magazine-papalter</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="2">
@@ -1783,14 +1783,14 @@
       </c>
       <c r="G46" t="inlineStr" s="2">
         <is>
-          <t>‘OJAT' 21' EDITORIAL</t>
+          <t>VISUAL for ‘In the Name of Love’ EDITORIAL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr" s="2">
         <is>
-          <t>ojat-lookbook-2021-development</t>
+          <t>ojat-magazine-babyyana</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="2">
@@ -1820,14 +1820,14 @@
       </c>
       <c r="G47" t="inlineStr" s="2">
         <is>
-          <t>‘OJAT' 21' DEVELOPMENT</t>
+          <t>OJAT for BABY YANA @M/V</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr" s="2">
         <is>
-          <t>ojat-lookbook-2020</t>
+          <t>ojat-magazine-yunwhay</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="2">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="E48" t="inlineStr" s="2">
         <is>
-          <t>2020</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="2">
@@ -1857,14 +1857,14 @@
       </c>
       <c r="G48" t="inlineStr" s="2">
         <is>
-          <t>‘OJAT' 20’ LOOKBOOK</t>
+          <t>OJAT for YUNWHAY</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr" s="2">
         <is>
-          <t>ojat-lookbook-2020-editorial</t>
+          <t>ojat-magazine-chorong</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="2">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E49" t="inlineStr" s="2">
         <is>
-          <t>2020</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="2">
@@ -1894,14 +1894,14 @@
       </c>
       <c r="G49" t="inlineStr" s="2">
         <is>
-          <t>‘OJAT' 20’ EDITORIAL</t>
+          <t>OJAT for Chorong(Apink)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr" s="2">
         <is>
-          <t>ojat-lookbook-2020-development</t>
+          <t>ojat-magazine-nain</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="2">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="E50" t="inlineStr" s="2">
         <is>
-          <t>2020</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="2">
@@ -1931,14 +1931,14 @@
       </c>
       <c r="G50" t="inlineStr" s="2">
         <is>
-          <t>‘OJAT' 20' DEVELOPMENT</t>
+          <t>OJAT for NAIN @BREAK MAGAZINE</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-pap</t>
+          <t>ojat-magazine-schön</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="2">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="E51" t="inlineStr" s="2">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="2">
@@ -1968,14 +1968,14 @@
       </c>
       <c r="G51" t="inlineStr" s="2">
         <is>
-          <t>VISAUL for 'PAP Magazine' - In the Name of Love</t>
+          <t>OJAT for SCHÖN! MAGAZINE</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-papalter</t>
+          <t>ojat-magazine-yena</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="2">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="E52" t="inlineStr" s="2">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="2">
@@ -2005,14 +2005,14 @@
       </c>
       <c r="G52" t="inlineStr" s="2">
         <is>
-          <t>VISUAL for ‘In the Name of Love’ EDITORIAL</t>
+          <t>OJAT for YENA @MAPS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-babyyana</t>
+          <t>ojat-magazine-jerd</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="2">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E53" t="inlineStr" s="2">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="2">
@@ -2042,14 +2042,14 @@
       </c>
       <c r="G53" t="inlineStr" s="2">
         <is>
-          <t>OJAT for BABY YANA @M/V</t>
+          <t>OJAT for JERD @NAVER ONstage</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-yunwhay</t>
+          <t>ojat-magazine-ugg</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="2">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="E54" t="inlineStr" s="2">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="2">
@@ -2079,14 +2079,14 @@
       </c>
       <c r="G54" t="inlineStr" s="2">
         <is>
-          <t>OJAT for YUNWHAY</t>
+          <t>OJAT for UGG &amp; AGE @shinsegae</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-chorong</t>
+          <t>ojat-magazine-bomi</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="2">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="E55" t="inlineStr" s="2">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="2">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="G55" t="inlineStr" s="2">
         <is>
-          <t>OJAT for Chorong(Apink)</t>
+          <t>OJAT for BOMI(Apink) @MAPS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-nain</t>
+          <t>ojat-magazine-breakmag</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="2">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="E56" t="inlineStr" s="2">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="2">
@@ -2153,14 +2153,14 @@
       </c>
       <c r="G56" t="inlineStr" s="2">
         <is>
-          <t>OJAT for NAIN @BREAK MAGAZINE</t>
+          <t>OJAT for BREAK MAGAZINE</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-schön</t>
+          <t>ojat-magazine-cakemag</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="2">
@@ -2190,14 +2190,14 @@
       </c>
       <c r="G57" t="inlineStr" s="2">
         <is>
-          <t>OJAT for SCHÖN! MAGAZINE</t>
+          <t>OJAT for CAKE MAGAZINE</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-yena</t>
+          <t>poster-2026-kyuto31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="2">
@@ -2207,17 +2207,17 @@
       </c>
       <c r="C58" t="inlineStr" s="2">
         <is>
-          <t>OJAT</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="D58" t="inlineStr" s="2">
         <is>
-          <t>Fashion</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="E58" t="inlineStr" s="2">
         <is>
-          <t>2022</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="2">
@@ -2227,14 +2227,14 @@
       </c>
       <c r="G58" t="inlineStr" s="2">
         <is>
-          <t>OJAT for YENA @MAPS</t>
+          <t>BIRTHDAY VISUALS for KYUTO</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-jerd</t>
+          <t>poster-2025-kyuto30</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="2">
@@ -2244,17 +2244,17 @@
       </c>
       <c r="C59" t="inlineStr" s="2">
         <is>
-          <t>OJAT</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="D59" t="inlineStr" s="2">
         <is>
-          <t>Fashion</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="E59" t="inlineStr" s="2">
         <is>
-          <t>2022</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="2">
@@ -2264,14 +2264,14 @@
       </c>
       <c r="G59" t="inlineStr" s="2">
         <is>
-          <t>OJAT for JERD @NAVER ONstage</t>
+          <t>BIRTHDAY VISUALS for KYUTO</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-ugg</t>
+          <t>poster-2025-hanni</t>
         </is>
       </c>
       <c r="B60" t="inlineStr" s="2">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="C60" t="inlineStr" s="2">
         <is>
-          <t>OJAT</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="D60" t="inlineStr" s="2">
         <is>
-          <t>Fashion</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="E60" t="inlineStr" s="2">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="2">
@@ -2301,14 +2301,14 @@
       </c>
       <c r="G60" t="inlineStr" s="2">
         <is>
-          <t>OJAT for UGG &amp; AGE @shinsegae</t>
+          <t>BIRTHDAY VISUALS for JONGIN</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-bomi</t>
+          <t>album-cover-lack</t>
         </is>
       </c>
       <c r="B61" t="inlineStr" s="2">
@@ -2318,17 +2318,17 @@
       </c>
       <c r="C61" t="inlineStr" s="2">
         <is>
-          <t>OJAT</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="D61" t="inlineStr" s="2">
         <is>
-          <t>Fashion</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="E61" t="inlineStr" s="2">
         <is>
-          <t>2022</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="2">
@@ -2338,14 +2338,14 @@
       </c>
       <c r="G61" t="inlineStr" s="2">
         <is>
-          <t>OJAT for BOMI(Apink) @MAPS</t>
+          <t>ALBUM COVER for LACK</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-breakmag</t>
+          <t>album-cover-crane</t>
         </is>
       </c>
       <c r="B62" t="inlineStr" s="2">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="C62" t="inlineStr" s="2">
         <is>
-          <t>OJAT</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="2">
         <is>
-          <t>Fashion</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="E62" t="inlineStr" s="2">
         <is>
-          <t>2022</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F62" t="inlineStr" s="2">
@@ -2375,34 +2375,34 @@
       </c>
       <c r="G62" t="inlineStr" s="2">
         <is>
-          <t>OJAT for BREAK MAGAZINE</t>
+          <t>ALBUM COVER for CRANE</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr" s="2">
         <is>
-          <t>ojat-magazine-cakemag</t>
+          <t>album-cover-laegyu</t>
         </is>
       </c>
       <c r="B63" t="inlineStr" s="2">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C63" t="inlineStr" s="2">
         <is>
-          <t>OJAT</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="D63" t="inlineStr" s="2">
         <is>
-          <t>Fashion</t>
+          <t>GRAPHIC</t>
         </is>
       </c>
       <c r="E63" t="inlineStr" s="2">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="2">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="G63" t="inlineStr" s="2">
         <is>
-          <t>OJAT for CAKE MAGAZINE</t>
+          <t>ALBUM COVER for LAEGYU</t>
         </is>
       </c>
     </row>

</xml_diff>